<commit_message>
Site: map-led Next.js report (county map, rep rulers, call-plan worksheet, balance, limits); workbook recoloured; 42 unit and 27 browser tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Field-Force-Sizing-Model.xlsx
+++ b/excel/Field-Force-Sizing-Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\claude-workspace\field-force\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F322755D-77C3-4FAE-81D5-3DEFABF45E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7CD1BE-DC22-4794-85F3-B2CDEEAC58B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -681,7 +681,7 @@
     <font>
       <b/>
       <sz val="14"/>
-      <color rgb="FF6D4C9F"/>
+      <color rgb="FF15302C"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -697,7 +697,7 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FF6D4C9F"/>
+      <color rgb="FF15302C"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -712,7 +712,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF6D6"/>
+        <fgColor rgb="FFF8EBA9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -733,16 +733,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFE6D9A8"/>
+        <color rgb="FF978429"/>
       </left>
       <right style="thin">
-        <color rgb="FFE6D9A8"/>
+        <color rgb="FF978429"/>
       </right>
       <top style="thin">
-        <color rgb="FFE6D9A8"/>
+        <color rgb="FF978429"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE6D9A8"/>
+        <color rgb="FF978429"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1420,7 +1420,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
-    <tabColor rgb="FF6D4C9F"/>
+    <tabColor rgb="FF15302C"/>
   </sheetPr>
   <dimension ref="B1:G18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1649,7 +1649,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
-    <tabColor rgb="FF6D4C9F"/>
+    <tabColor rgb="FF15302C"/>
   </sheetPr>
   <dimension ref="A1:H57"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>